<commit_message>
paradox catalog complete: 46/46 cards + SHOWCASE alignment + neutrality masters
- AR working journal: full record of the catalog pass -- all 46 paradox
  cards expanded (13 structural, 25 defective, 8 non-paradoxes) with
  per-card domain analysis D1-D6, E/R/R diagnosis, dissolution/resolution
  and honest machine anchors; paradox generation detached in catalog2md.ps1
- docs/SHOWCASE.md/.tex/.pdf: "postulates" -> "tool assumptions" wording
  in 6 places, PDF rebuilt (25 pp)
- tools/md2tex.ps1 + tools/showcase_md2tex.ps1: SHOWCASE build pipeline
- docs/logical_fallacies_classification (3).xlsx: master synced with 71
  neutral example replacements (TSV pass)
- docs/paradoxes_classification_v4.xlsx: paradox table master (46 entries)

Site content itself (cards, catalog indexes, Formalization page) lives in
the quartz working copy and the site/quartz mirror (untracked by precedent).

Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/logical_fallacies_classification (3).xlsx
+++ b/docs/logical_fallacies_classification (3).xlsx
@@ -131,7 +131,7 @@
     <t>Условия нарушены: часть пространства аргументов априори закрыта. Рассуждение не может начаться честно.</t>
   </si>
   <si>
-    <t>«Не обсуждаем моё пьянство»; «Не смей играть расовую карту»; «против Библии»</t>
+    <t>«Не обсуждаем моё пьянство»; «эту тему в семье не поднимают»</t>
   </si>
   <si>
     <t>2.6.4.7, 3.2.1, 2.6.4.2</t>
@@ -164,7 +164,7 @@
     <t>Условия нарушены произвольно: аргумент не рассматривается из-за контекста.</t>
   </si>
   <si>
-    <t>«Facebook не место для политики»; «Это неподходящий форум» — когда проигрываешь</t>
+    <t>«Рабочий чат — не место для этого вопроса»; «Это неподходящий форум» — когда проигрываешь</t>
   </si>
   <si>
     <t>Disciplinary Blinders, 1.A.4</t>
@@ -203,7 +203,7 @@
     <t>Рассуждение полностью подменяется принуждением. Сила не доказывает правоту. «Соглашайся или пострадаешь» — это не аргумент, а угроза.</t>
   </si>
   <si>
-    <t>«Отдай кошелёк или получишь по голове»; «У нас большие пушки — значит, эта земля наша»</t>
+    <t>«Отдай кошелёк или получишь по голове»; «Или подписываешь, или уволен»</t>
   </si>
   <si>
     <t>1.B.10</t>
@@ -257,7 +257,7 @@
     <t>Рассуждение отвергается в принципе. Оппонент изображается как монстр, лишённый разума. Сила подменяет аргумент.</t>
   </si>
   <si>
-    <t>«На землю, немедленно!»; «Настоящий лидер не извиняется — только стреляет»</t>
+    <t>«Обсуждать нечего — делай, как сказано»; «Кто спорит — тот против нас»</t>
   </si>
   <si>
     <t>1.B.1.1, 2.3.6.3</t>
@@ -314,7 +314,7 @@
     <t>Рассуждение прерывается односторонне: отказ продолжать как форма давления. Пассивно-агрессивная тактика.</t>
   </si>
   <si>
-    <t>Бойкоты, забастовки как давление; полувековой отказ США от диалога с Кубой</t>
+    <t>Бойкоты, забастовки как давление; сосед годами не здоровается после спора о заборе</t>
   </si>
   <si>
     <t>1.B.1.3, 2.6.4.8</t>
@@ -617,7 +617,7 @@
     <t>Рассуждение подменяется сознательным обманом: говорящий знает, что его аргумент ложен. Включает «мотивационную правду» — ложь для «благой цели».</t>
   </si>
   <si>
-    <t>Адвокат защищает клиента, которого знает виновным; неверующий атакует верующих цитатами из их писаний</t>
+    <t>Адвокат защищает клиента, которого знает виновным; спорщик отстаивает позицию, в которую сам не верит, ради победы</t>
   </si>
   <si>
     <t>1.B.8, Self Deception</t>
@@ -650,7 +650,7 @@
     <t>Манипуляция процессом: информация подаётся в момент, когда оппонент не может ответить. Запрещено в судах.</t>
   </si>
   <si>
-    <t>«Ой, забыл: вас ведь уже дважды судили за это?!» — в конце процесса; «October Surprise»</t>
+    <t>«Ой, забыл: вас ведь уже дважды судили за это?!» — в конце процесса; внезапное «вспомнил» в конце переговоров</t>
   </si>
   <si>
     <t>1.B.14, 1.B.8</t>
@@ -743,7 +743,7 @@
     <t>Рассуждение подменяется избирательным патосом: показывают только «правильных» жертв для обоснования интервенции.</t>
   </si>
   <si>
-    <t>Дети рохинджа (но не других этносов); дети в повстанческих районах (но не правительственных)</t>
+    <t>«Спасём детей нашего двора!» — о детях соседнего молчание; жалость по списку</t>
   </si>
   <si>
     <t>1.B.2, 2.1.3</t>
@@ -773,7 +773,7 @@
     <t>Рассуждение подменяется триггером: короткая фраза вызывает немедленную эмоциональную реакцию, минуя анализ. Попытка деконструировать триггер встречает ярость или недоумение.</t>
   </si>
   <si>
-    <t>Политические дебаты, где участники «свистят» триггерные слова своей аудитории вместо рассмотрения аргументов</t>
+    <t>Выступающий «свистит» словечки-сигналы своей аудитории вместо рассмотрения аргументов</t>
   </si>
   <si>
     <t>1.B.3, Reductionism</t>
@@ -800,7 +800,7 @@
     <t>Рассуждение подменяется эмоциональным воздействием: шок, возмущение или идентификация через язык. Нецензурность не делает аргумент сильнее.</t>
   </si>
   <si>
-    <t>Добавление «взрослых» сцен в фильм только для избежания рейтинга G; сексуализация политической критики</t>
+    <t>Добавление «взрослых» сцен в фильм только ради рейтинга; скабрёзность вместо довода</t>
   </si>
   <si>
     <t>1.B.3, Red Herring</t>
@@ -860,7 +860,7 @@
     <t>Рассуждение подменяется патосом: имена создают мистическое воздействие, но это не аргумент.</t>
   </si>
   <si>
-    <t>Зачитывание имён жертв 9/11; списки погибших на мемориалах</t>
+    <t>Зачитывание длинного списка подписей «против» вместо довода — вес числа вместо разбора</t>
   </si>
   <si>
     <t>1.B.2, 1.B.2.2</t>
@@ -890,7 +890,7 @@
     <t>Рассуждение подменяется страхом: паника используется для протаскивания неприемлемых решений.</t>
   </si>
   <si>
-    <t>«Если не сделаете как я говорю — умрём!»; «Это о безопасности!»; Patriot Act после 9/11</t>
+    <t>«Если не сделаете как я говорю — всё пропало!»; продавец сигнализаций открывает разговор сводкой краж</t>
   </si>
   <si>
     <t>1.B.3.3, Shock Doctrine</t>
@@ -920,7 +920,7 @@
     <t>Рассуждение подменяется эмоциональным состоянием: решения «в жару момента».</t>
   </si>
   <si>
-    <t>Patriot Act и Homeland Security — Америка «покупала голодной» после 9/11</t>
+    <t>После кражи в подъезде дом закупил самую дорогую охрану, ничего не сравнив, — покупка «на голодный желудок»</t>
   </si>
   <si>
     <t>1.B.3.5, 2.3.6.1</t>
@@ -998,7 +998,7 @@
     <t>Уничтожается само условие рассуждения — различие истины и лжи. Если это различие не существует, рассуждение невозможно в принципе. Атака на фундамент.</t>
   </si>
   <si>
-    <t>Настаивание на «альтернативных фактах», противоречащих задокументированной реальности</t>
+    <t>Настаивание на своей версии вопреки задокументированной реальности</t>
   </si>
   <si>
     <t>4.2</t>
@@ -1028,7 +1028,7 @@
     <t>Рассуждение подменяется повторением. Ложь не становится истиной от повторения, но начинает восприниматься как «уже известный факт». Чем наглее ложь, тем она убедительнее.</t>
   </si>
   <si>
-    <t>«Еврейский вопрос» — не было никакого еврейского вопроса. «Оружие массового поражения в Ираке» — не существовало.</t>
+    <t>«Еврейский вопрос» нацистской пропаганды — не было никакого «вопроса»; ложь, слишком большая, чтобы её заподозрить, повторяется до привычности.</t>
   </si>
   <si>
     <t>1.B.8, 2.3.5.5, 2.1.1</t>
@@ -1055,7 +1055,7 @@
     <t>Атака на саму возможность рассуждения: подрывается доверие к собственному восприятию и памяти. «Кому ты веришь — мне или своим глазам?»</t>
   </si>
   <si>
-    <t>«Ты утверждаешь, что застала меня с ней в постели? Ты сумасшедшая! Тебе нужен психиатр»</t>
+    <t>«Ты же видела счёт своими глазами? Тебе показалось — ты вечно всё путаешь и выдумываешь»</t>
   </si>
   <si>
     <t>1.B.8.1, 1.B.12</t>
@@ -1082,7 +1082,7 @@
     <t>Разрушение условий рассуждения: граница между фактом и вымыслом размывается намеренно. Аудитория не может отличить новость от развлечения.</t>
   </si>
   <si>
-    <t>Жёлтая пресса; «InfoWars»; смешение новостей и развлечений с оговоркой «только для развлечения»</t>
+    <t>Жёлтая пресса; смешение новостей и развлечений с оговоркой «только для развлечения»</t>
   </si>
   <si>
     <t>1.B.8.1, 1.B.3.1</t>
@@ -1115,7 +1115,7 @@
     <t>Рассуждение подменяется повторением скриптов: не диалог, а трансляция заготовок для эффекта.</t>
   </si>
   <si>
-    <t>Политики повторяют одни фразы независимо от вопроса; talking points вместо ответа</t>
+    <t>Пресс-секретарь повторяет одни фразы независимо от вопроса; заготовки вместо ответа</t>
   </si>
   <si>
     <t>1.B.8.1, Dog Whistle</t>
@@ -1148,7 +1148,7 @@
     <t>Рассуждение подменяется ссылкой на непроверяемый авторитет. «Бог велел» делает невозможным ни проверку, ни возражение. Отказ от рассуждения через апелляцию к абсолюту.</t>
   </si>
   <si>
-    <t>«Бог велел мне убить детей»; «Эта земля дана нам Богом, дальнейшее обсуждение излишне»</t>
+    <t>«Так угодно небу — обсуждение излишне»; «Высшая воля на нашей стороне — спорить не о чем»</t>
   </si>
   <si>
     <t>2.6.4</t>
@@ -1187,7 +1187,7 @@
     <t>Подмена объекта: вместо темы (A) вводится другая (A'), эмоциональная, но не связанная.</t>
   </si>
   <si>
-    <t>«Насчёт моих банкротств — давайте о терроризме!»; «BLM» → «Climate Change Matters»</t>
+    <t>«Про мой отчёт — а вы видели, что творится у соседей?» — разговор уведён прочь</t>
   </si>
   <si>
     <t>2.1.3.1, Dog Whistle</t>
@@ -1214,7 +1214,7 @@
     <t>Деформация: реальный аргумент заменяется карикатурой. Побеждается не позиция, а её искажение.</t>
   </si>
   <si>
-    <t>«Вегетарианцы говорят о чувствах — видели корову над Шекспиром?»; «Pro-choice ненавидят детей»</t>
+    <t>«Вегетарианцы говорят о чувствах — видели корову над Шекспиром?»; «Сторонники удалёнки хотят развалить компанию»</t>
   </si>
   <si>
     <t>2.1.1.1, 2.1.2.8</t>
@@ -1358,7 +1358,7 @@
     <t>Замена объекта: вместо оценки аргумента — авторитет знаменитости. Включает цитирование вне контекста.</t>
   </si>
   <si>
-    <t>«Олимпийский чемпион использует X — а вы?»; «Рок-звезда против вакцин»</t>
+    <t>«Олимпийский чемпион использует X — а вы?»; звезда рекламирует диету, в которой не разбирается</t>
   </si>
   <si>
     <t>Является ли эта знаменитость экспертом в данной области?</t>
@@ -1442,7 +1442,7 @@
     <t>Замена объекта: вместо защиты позиции — атака на оппонента. «Ты тоже» не делает действие правильным.</t>
   </si>
   <si>
-    <t>«Да, мы пытали, но мы не отрезаем головы!»; Трамп: «Путин убийца? У нас тоже»</t>
+    <t>«Да, я опоздал — а ты вчера вообще не пришёл!»; «Сам-то отчёт сдал с ошибками!»</t>
   </si>
   <si>
     <t>2.1.1.1, 2.1.2.1</t>
@@ -1472,7 +1472,7 @@
     <t>Замена объекта: вместо аргумента (A) рассматриваются мотивы говорящего (B). Но даже злые люди иногда говорят правду, а добрые — ошибаются. Мотив не определяет истинность.</t>
   </si>
   <si>
-    <t>«Бен Ладен хотел, чтобы мы ушли из Афганистана, значит мы должны остаться»</t>
+    <t>«Конкурент хочет, чтобы мы ушли с рынка, — значит, остаёмся» — решение от чужого желания, не от расчёта</t>
   </si>
   <si>
     <t>2.1.2.1, 1.B.6</t>
@@ -1523,7 +1523,7 @@
     <t>Замена объекта: вместо аргумента (A) оценивается групповая принадлежность говорящего (B). Партийность не определяет истинность.</t>
   </si>
   <si>
-    <t>«Не слушай её, она республиканка»; «Ты был в Коммунистической партии?»</t>
+    <t>«Не слушай его — он из той самой конторы»; «Ты дружил с этим человеком?»</t>
   </si>
   <si>
     <t>2.1.2.1, 2.1.2.2</t>
@@ -1550,7 +1550,7 @@
     <t>Замена объекта: вместо аргумента (A) оценивается идентичность говорящего (B). Аргументы отвергаются без рассмотрения по существу.</t>
   </si>
   <si>
-    <t>«Ты бы понял, если бы был бирманцем, но раз нет — объяснять бесполезно»</t>
+    <t>«Ты бы понял, если бы работал в нашем цеху, а раз нет — объяснять бесполезно»</t>
   </si>
   <si>
     <t>2.1.2.1, 2.1.2.4, Othering</t>
@@ -1577,7 +1577,7 @@
     <t>Замена объекта: вместо аргумента (A) оценивается имидж говорящего как «своего» (B). «Он простой парень» — не доказывает истинность.</t>
   </si>
   <si>
-    <t>Политик позиционирует себя как «простого человека» в противовес «элите», «профессорам»</t>
+    <t>Кандидат в правление дома зовёт себя «простым жильцом» в противовес «умникам» и «профессорам»</t>
   </si>
   <si>
     <t>2.1.2.1, 2.1.2.5</t>
@@ -1631,7 +1631,7 @@
     <t>Замена объекта: вместо аргументов оценивается воображаемый запах оппонента. Дегуманизация через отвращение.</t>
   </si>
   <si>
-    <t>«Поговорю с демонстрантами, когда помоются»; «Я чувствую еврея за квартал»</t>
+    <t>«Поговорю с вами, когда будете выглядеть прилично»; «От этого предложения дурно пахнет» — вместо разбора</t>
   </si>
   <si>
     <t>2.1.2.1, Othering</t>
@@ -1658,7 +1658,7 @@
     <t>Замена объекта: вместо аргументов оценивается принадлежность к «чужой» группе. Крайняя форма — дегуманизация.</t>
   </si>
   <si>
-    <t>«Для мексиканцев нормально зарабатывать доллар в час — они не такие»; «террористы иначе относятся к смерти»</t>
+    <t>«Стажёрам отдых не нужен — молодые, привыкли»; «у них всё иначе — с ними нельзя как с нами»</t>
   </si>
   <si>
     <t>2.1.2.5, 2.1.2.7, Dehumanization</t>
@@ -1745,7 +1745,7 @@
     <t>Фильтрация: каждый отдельный факт истинен, но целое ложно из-за намеренных упущений. Правда сказана, но важное скрыто.</t>
   </si>
   <si>
-    <t>Описание Бангладеш как райского места с умолчанием о бедности, перенаселении, наводнениях</t>
+    <t>Объявление о квартире: «солнечная сторона, тихие соседи» — с умолчанием о трассе под окнами</t>
   </si>
   <si>
     <t>2.1.3.1, 4.1</t>
@@ -1802,7 +1802,7 @@
     <t>Фильтрация: проблема игнорируется, если физически удалена или скрыта из медиа. Проблема не решена — только перемещена.</t>
   </si>
   <si>
-    <t>«Построить стену»; отправить проблему в Гуантанамо; переместить бездомных в другой район</t>
+    <t>«Свалка городу нужна — но не на нашей улице»; проблему не решают — переносят к другим</t>
   </si>
   <si>
     <t>2.1.3.1, 2.6.4.3</t>
@@ -1835,7 +1835,7 @@
     <t>Проекция: собственные интерпретации чужих мыслей принимаются за факт. Спекуляция выдаётся за знание.</t>
   </si>
   <si>
-    <t>«Обама на самом деле плевать хотел на права человека» — безосновательное утверждение о мотивах</t>
+    <t>«Начальнику на самом деле плевать на команду» — безосновательное утверждение о чужих мотивах</t>
   </si>
   <si>
     <t>2.1.4, 2.1.2.2</t>
@@ -1862,7 +1862,7 @@
     <t>Проекция: свои ценности приписываются другим без проверки. Отрицает реальность различий и способность к злу.</t>
   </si>
   <si>
-    <t>«Нацисты хотели мира и семьи, как мы» (реальность иная); «Хамас хочет сосуществования»</t>
+    <t>«Все ведь хотят того же, что и мы» — свои мотивы спроецированы на другую сторону переговоров</t>
   </si>
   <si>
     <t>2.1.2.9, 2.1.4.1</t>
@@ -1985,7 +1985,7 @@
     <t>Термин сознательно используется в двух значениях: говорящий имеет в виду одно, аудитория понимает другое. Формально «не солгал», фактически — обманул.</t>
   </si>
   <si>
-    <t>Клинтон: «У меня не было сексуальных отношений с этой женщиной» (имея в виду только проникновение)</t>
+    <t>«Ничего нет лучше истины; бутерброд лучше, чем ничего, — значит, бутерброд лучше истины» — «ничего» меняет смысл посреди хода</t>
   </si>
   <si>
     <t>2.2.1.1, 2.2.2</t>
@@ -2093,7 +2093,7 @@
     <t>Абстракция принимается за реальность: категория становится «вещью». Карта путается с территорией.</t>
   </si>
   <si>
-    <t>«Война с террором — борьба Свободы против Абсолютного Зла!»</t>
+    <t>«Рынок решил»; «Наука говорит» — абстракции, взятые деятелями</t>
   </si>
   <si>
     <t>2.6.1.3, 2.2.1</t>
@@ -2129,7 +2129,7 @@
     <t>Неполное прояснение: кто действует — скрыто. «Было решено вас уволить» вместо «я решил». Ответственность размывается.</t>
   </si>
   <si>
-    <t>«Сколько женщин было изнасиловано» вместо «сколько мужчин изнасиловали»; «Насилие над женщинами»</t>
+    <t>«Были допущены ошибки» вместо «мы ошиблись»; «ваза разбилась» вместо «я разбил» — деятель спрятан залогом</t>
   </si>
   <si>
     <t>Political Correctness, 2.1.2</t>
@@ -2162,7 +2162,7 @@
     <t>Пространство возможностей не исследовано: из множества вариантов представлены только два крайних. Промежуточные и альтернативные варианты игнорируются.</t>
   </si>
   <si>
-    <t>«Либо ты на 100% с нами, либо ты враг!»; Противопоставление «Black Lives Matter» и «Blue Lives Matter»</t>
+    <t>«Либо ты на 100% с нами, либо ты враг!»; «Ты за качество или за скорость?» — будто третьего не дано</t>
   </si>
   <si>
     <t>1.A.4, 2.5.4</t>
@@ -2504,7 +2504,7 @@
     <t>Рамка оценки: «древность/традиционность = правильность». Длительность практики не связана с её истинностью или моральной оправданностью. Рабство тоже было традицией.</t>
   </si>
   <si>
-    <t>«В Америке женщинам всегда платили меньше, так что не будем нарушать давнюю традицию»</t>
+    <t>«У нас всегда вели учёт в тетради — не будем нарушать давнюю традицию»</t>
   </si>
   <si>
     <t>2.3.5.3, 2.6.3.1</t>
@@ -2639,7 +2639,7 @@
     <t>Нерелевантный критерий: «выполнял приказы» ≠ «заслуживает чести». Опровергнуто в Нюрнберге.</t>
   </si>
   <si>
-    <t>Почитание солдат Гитлера, Сталина наравне с защитниками свободы; «он делал работу»</t>
+    <t>Почитание исполнителей любой стороны «за службу» — без вопроса, какому делу служили; «он просто делал работу»</t>
   </si>
   <si>
     <t>2.6.4.4, 2.2.1.5, 1.B.12</t>
@@ -2816,7 +2816,7 @@
     <t>Ложная аналогия: война или интимность — не игра с «очками». Спортивная рамка скрывает реальные ставки.</t>
   </si>
   <si>
-    <t>«Ещё не забил с Фрэнсис, но дошёл до третьей базы»; «перенести игру на поле Кима»</t>
+    <t>«Мы порвали конкурентов в финале переговоров» — спортивная лексика там, где не спорт</t>
   </si>
   <si>
     <t>2.4.1.1, 2.3.1</t>
@@ -2993,7 +2993,7 @@
     <t>Сравнение реального человека с недостижимым идеалом. Любое отклонение от совершенства используется для полной дисквалификации.</t>
   </si>
   <si>
-    <t>«Вашингтон держал рабов, Линкольн был расистом, Кинг изменял жене — героев не существует»</t>
+    <t>«У каждого мастера найдётся брак — значит, мастеров не существует»</t>
   </si>
   <si>
     <t>2.4.5, 2.2.3.1</t>
@@ -3062,7 +3062,7 @@
     <t>Ложная причинность: из несчастья выводится вина. «Случилось плохое → кто-то согрешил». Причинная связь постулируется без механизма.</t>
   </si>
   <si>
-    <t>Церковь Вестборо протестует на похоронах солдат: смерть — наказание за грехи Америки</t>
+    <t>«Сам виноват — к живущим правильно беда не приходит»: страдание прочитано как приговор</t>
   </si>
   <si>
     <t>1.B.9, Magical Thinking</t>
@@ -3089,7 +3089,7 @@
     <t>Ложная причинность: вера/ритуал → желаемый результат. Причинная связь постулируется без механизма. Отрицание предсказуемой вселенной.</t>
   </si>
   <si>
-    <t>«Назови это и потребуй» — если достаточно верить и молиться, Бог совершит чудо</t>
+    <t>«Загадай правильно — и вселенная услышит»; ритуал перед экзаменом вместо подготовки</t>
   </si>
   <si>
     <t>1.B.9, 2.5.2.1</t>
@@ -3170,7 +3170,7 @@
     <t>Ложная причинность: временнáя последовательность ≠ причинная связь. Корреляция ≠ каузация.</t>
   </si>
   <si>
-    <t>«СПИД появился вместе с диско — диско вызвало СПИД!»</t>
+    <t>«Петух прокукарекал — и солнце взошло: значит, поднял!»</t>
   </si>
   <si>
     <t>2.5.2, Clustering Illusion</t>
@@ -3200,7 +3200,7 @@
     <t>Ложная причинность: вина приписывается не реальному источнику, а удобной цели. Включает «обвинение жертвы».</t>
   </si>
   <si>
-    <t>«Евреи виноваты!»; «Ты сама виновата в изнасиловании — флиртовала»</t>
+    <t>«Во всех сбоях виноват новый отдел!»; «Сам виноват, что тебя обманули»</t>
   </si>
   <si>
     <t>2.5.2, Affective Fallacy</t>
@@ -3293,7 +3293,7 @@
     <t>Цепочка не обоснована: каждый переход требует доказательства, но выдаётся за неизбежность.</t>
   </si>
   <si>
-    <t>«Кофе вместе → беременность → welfare»; «Закроем Гуантанамо → террористы в церквях Канзаса»</t>
+    <t>«Разрешишь телефон за ужином → забросит учёбу → останется без работы» — каждое звено выдано за неизбежное</t>
   </si>
   <si>
     <t>2.5.3.1, 2.5.2</t>
@@ -3329,7 +3329,7 @@
     <t>Вывод об истинности делается из нежелательности последствий. Но желательность/нежелательность последствий не влияет на истинность посылок. «Мне не нравится вывод» ≠ «посылка ложна».</t>
   </si>
   <si>
-    <t>«Изменение климата не может быть вызвано человеком, потому что тогда придётся перестраивать всю экономику»</t>
+    <t>«Диагноз не может быть верным — иначе придётся перестраивать всю жизнь»</t>
   </si>
   <si>
     <t>Влияет ли нежелательность последствий на истинность утверждения?</t>
@@ -3353,7 +3353,7 @@
     <t>Вывод из нереалистичной посылки: худший сценарий принимается за вероятный.</t>
   </si>
   <si>
-    <t>«Что если террористы атакуют зернохранитель? Запасайтесь оружием!»</t>
+    <t>«А если метеорит в склад? Готовимся ко всему разом!»</t>
   </si>
   <si>
     <t>1.B.3.5, 2.5.2.4</t>
@@ -3380,7 +3380,7 @@
     <t>Отсутствие доказательства принимается за доказательство отсутствия (или наоборот). Вывод превышает основание: из «не знаем» не следует ни «да», ни «нет».</t>
   </si>
   <si>
-    <t>«Учёные не могут доказать эволюцию, потому что нас там не было. Значит, буквальное творение за 6 дней — истина!»</t>
+    <t>«Никто не доказал, что чудовища в озере нет. Значит, оно есть!»</t>
   </si>
   <si>
     <t>2.2.3, 3.2.1</t>
@@ -3407,7 +3407,7 @@
     <t>Вывод превышает основание: из отсутствия информации делается положительный вывод. «Источники молчат о X» ≠ «X истинно/ложно». Молчание не является доказательством.</t>
   </si>
   <si>
-    <t>«Мистер Хиксон не может предоставить алиби. Это доказывает, что он был в комнате 331 и убивал жену топором!»</t>
+    <t>«Он не может сказать, где был вечером. Значит, витрину разбил он!» — молчание прочитано как улика</t>
   </si>
   <si>
     <t>Является ли молчание/отсутствие данных доказательством чего-либо?</t>
@@ -3431,7 +3431,7 @@
     <t>Вывод формально не делается, но провоцируется. Данные подобраны так, чтобы вывод казался «очевидным». Аудитория делает вывод, превышающий основание, но чувствует его «своим».</t>
   </si>
   <si>
-    <t>«Уровень преступности среди группы X вдвое выше среднего — делайте выводы сами»</t>
+    <t>«Тот отдел снова сорвал сроки — выводы делайте сами»</t>
   </si>
   <si>
     <t>2.1.3, 1.A.2</t>
@@ -3461,7 +3461,7 @@
     <t>Вывод превышает основание: из «очень маловероятно» не следует «невозможно». Низкая вероятность ≠ нулевая. При достаточном времени маловероятные события случаются.</t>
   </si>
   <si>
-    <t>«Вероятность появления ДНК случайно так мала, что это невозможно — значит, было божественное вмешательство»</t>
+    <t>«Вероятность такой раздачи карт ничтожна — колода подстроена!» — а какая-то раздача выпадает всегда</t>
   </si>
   <si>
     <t>2.6.4.1, 2.5.4.2</t>
@@ -3488,7 +3488,7 @@
     <t>Вывод превышает основания: из общего не следует игнорирование частного; из частного не следует целое. Включает Pars pro Toto.</t>
   </si>
   <si>
-    <t>«Black Lives Matter» → «All Lives Matter»; один преступник из меньшинства → «все они такие»</t>
+    <t>«Один курьер опоздал — все курьеры ненадёжны»; три первых лебедя белы — «все лебеди белы»</t>
   </si>
   <si>
     <t>2.5.4, Zero Tolerance</t>
@@ -3521,7 +3521,7 @@
     <t>Вывод без оснований: «молчаливое большинство» постулируется без доказательств. Вариант Argument from Ignorance.</t>
   </si>
   <si>
-    <t>Никсон о «молчаливом большинстве»; лидер как «голос безголосых»</t>
+    <t>«За меня — все, кто молчит: их большинство»; лидер как «голос безголосых»</t>
   </si>
   <si>
     <t>2.5.4.2, 2.5.4</t>
@@ -3548,7 +3548,7 @@
     <t>Вывод превышает основания: из слабых признаков делается сильный вывод. «Похоже» ≠ «является».</t>
   </si>
   <si>
-    <t>«Смуглый пассажир читает книгу со странными буквами — террорист!»</t>
+    <t>«Про него ходят слухи — что-то в них наверняка есть»</t>
   </si>
   <si>
     <t>2.6.1.6, Just in Case</t>
@@ -3620,7 +3620,7 @@
     <t>Рефлексия должна признавать границы и открытые вопросы. Требование «closure» закрывает рефлексию насильственно: вывод объявляется окончательным не потому, что обоснован, а потому что «нужна определённость».</t>
   </si>
   <si>
-    <t>«Общество было бы защищено пожизненным заключением, но нам нужна казнь, чтобы дать closure жертвам»</t>
+    <t>«Нужно окончательное решение — люди устали от вопроса»: завершённость вместо разбора по существу</t>
   </si>
   <si>
     <t>Является ли «потребность в closure» логическим основанием для вывода? Может ли вопрос оставаться открытым?</t>
@@ -3668,7 +3668,7 @@
     <t>Рефлексия закрыта: текущее состояние объявляется неизменной «сущностью» или «природой». Изменение объявляется невозможным a priori. Неопровергаемое утверждение.</t>
   </si>
   <si>
-    <t>«Все террористы — монстры и останутся монстрами до 100 лет»; «Бедные всегда будут с нами»</t>
+    <t>«Он лентяй по природе — не изменится»; «опоздун — это диагноз»</t>
   </si>
   <si>
     <t>2.6.1.2, 2.3.5.3</t>
@@ -3854,7 +3854,7 @@
     <t>Рефлексия блокируется sunk cost: прошлые инвестиции (усилия, жертвы, кровь) используются как аргумент против пересмотра решения. «Мы уже столько вложили» не является аргументом за правильность курса.</t>
   </si>
   <si>
-    <t>«Мы не можем вывести войска — тогда все погибшие солдаты погибли напрасно»</t>
+    <t>«Нельзя закрыть проект — иначе два года работы окажутся напрасными»</t>
   </si>
   <si>
     <t>2.6.3, 2.3.5.4, 2.5.4.1</t>
@@ -3935,7 +3935,7 @@
     <t>Рефлексия блокируется цинизмом: универсальное обвинение оправдывает бездействие. Круговая логика.</t>
   </si>
   <si>
-    <t>«Все политики жулики — зачем участвовать?»; «Все СМИ врут — зачем читать?»</t>
+    <t>«Все таксисты обманывают — зачем спрашивать цену?»; «Все врачи в сговоре — зачем ходить?»</t>
   </si>
   <si>
     <t>3.2, 2.6.4.3</t>
@@ -3962,7 +3962,7 @@
     <t>Рефлексия блокируется сверх-цинизмом: «меня не проведёшь» = отказ от любой информации.</t>
   </si>
   <si>
-    <t>Отказ от вакцин, потому что «врачи лгут»; игнорирование всех СМИ</t>
+    <t>«Реклама действует на всех, кроме меня» — и потому смотрю без защиты</t>
   </si>
   <si>
     <t>2.6.4.3, 2.4.1.3, 1.B.8.1</t>
@@ -3989,7 +3989,7 @@
     <t>Рефлексия блокируется: «я не это имел в виду» — хотя именно это и было сказано искренне.</t>
   </si>
   <si>
-    <t>«Это был просто разговор в раздевалке»; «альфа-самец так говорит»</t>
+    <t>«Я не всерьёз это сказал — просто сорвался»; «все так шутят»</t>
   </si>
   <si>
     <t>Affective Fallacy, 2.2.1.6</t>
@@ -4019,7 +4019,7 @@
     <t>Рефлексия отказывает в рассмотрении: валидные возражения заранее дисквалифицируются как «приём» или «карта». Вместо ответа на аргумент — метаобвинение в манипуляции.</t>
   </si>
   <si>
-    <t>«Не пытайся разыграть против меня расовую карту»; «Она опять достала свою женскую карту»</t>
+    <t>«Это ты давишь на жалость» — в ответ на реальную жалобу; обвинение в «карте» вместо разбора</t>
   </si>
   <si>
     <t>2.6.4.1, 2.1.2.1</t>
@@ -4100,7 +4100,7 @@
     <t>Рефлексия отклоняется: право говорить подменяет обоснованность сказанного. «Я имею право это сказать» ≠ «это правда». Свобода слова защищает от цензуры, не от критики.</t>
   </si>
   <si>
-    <t>«Я могу говорить что хочу!» — в ответ на просьбу обосновать; «Safe space» как защита от любых вопросов</t>
+    <t>«Я могу говорить что хочу!» — в ответ на просьбу обосновать</t>
   </si>
   <si>
     <t>2.6.4, 2.1.2</t>
@@ -4127,7 +4127,7 @@
     <t>Рефлексия блокируется ложной беспомощностью: «я ничего не могу сделать» закрывает обсуждение альтернатив. На самом деле власть есть.</t>
   </si>
   <si>
-    <t>«Что мы можем сделать с ценами на бензин? Как министр энергетики, я бы хотел иметь волшебную палочку...»</t>
+    <t>«Что делать с расходами? Как директор, я бы хотел иметь волшебную палочку...»</t>
   </si>
   <si>
     <t>Действительно ли нет возможности влияния? Или это способ избежать ответственности?</t>
@@ -4151,7 +4151,7 @@
     <t>Рефлексия блокируется ложной приватностью: критика отклоняется как вторжение в личное пространство.</t>
   </si>
   <si>
-    <t>«Да, я ехал 80 миль/час — тебе-то что? Ты не коп»; «Да, я убила ребёнка. И что? Не твоё дело»</t>
+    <t>«Да, я ехал 80 миль/час — тебе-то что? Ты не коп»; «Да, я нарушил регламент. И что? Не твоё дело»</t>
   </si>
   <si>
     <t>2.6.4, Taboo</t>
@@ -4181,7 +4181,7 @@
     <t>Рефлексия блокируется идеологией: факты не признаются, чтобы не «легитимизировать» врага. Реальность не исчезает от непризнания.</t>
   </si>
   <si>
-    <t>США десятилетиями не признавали КНР; отказ называть режим КНДР по имени</t>
+    <t>Фирма годами не называет конкурента по имени в отчётах — будто его нет</t>
   </si>
   <si>
     <t>2.6.4.3, 2.1.3.5</t>
@@ -4247,7 +4247,7 @@
     <t>Закон Порядка нарушен инверсией: вместо движения Д1→Д5 рассуждение идёт Д5→Д1. Вывод предшествует посылкам, посылки подбираются под вывод.</t>
   </si>
   <si>
-    <t>«Поскольку мы знаем, что эволюции не существует, наш долг — искать способы объяснить ДНК-данные, которые могли бы её подтверждать»</t>
+    <t>«Поскольку мы знаем, что наш прибор не ошибается, наша задача — объяснить, почему данные показывают иначе»</t>
   </si>
   <si>
     <t>4.1, 2.1.3, 3.2.2</t>
@@ -4385,7 +4385,7 @@
     <t>Нарушение закона противоречия: A и не-A истинны в разных «отсеках». «Знаю, но не верю».</t>
   </si>
   <si>
-    <t>Одно в науке, противоположное в религии; «предвыборная риторика» vs реальная политика</t>
+    <t>На экзамене отвечает по учебнику, в жизни действует наоборот — и разлада не замечает</t>
   </si>
   <si>
     <t>Disciplinary Blinders, 1.B.8.2</t>
@@ -4418,7 +4418,7 @@
     <t>Все домены искажаются в направлении подтверждения желаемого результата. Рационализация вместо рассуждения.</t>
   </si>
   <si>
-    <t>Инвестор находит причины держать убыточную акцию; верующий находит подтверждения своей веры везде</t>
+    <t>Инвестор находит причины держать убыточную акцию; болельщик находит судейский заговор в каждом матче</t>
   </si>
   <si>
     <t>4.1.1, 4.1.2</t>
@@ -4451,7 +4451,7 @@
     <t>Фильтрация данных (Д1) + выбор рамки (Д3) + отсутствие рефлексии (Д6) создают устойчивую систему.</t>
   </si>
   <si>
-    <t>Политические пузыри в соцсетях; секты; радикальные сообщества</t>
+    <t>Лента, собранная из одних единомышленников; клуб, где несогласных не осталось</t>
   </si>
   <si>
     <t>4.1.1, 2.1.3, 2.6.4.3</t>
@@ -4511,7 +4511,7 @@
     <t>Социальное давление блокирует рефлексию (Д6) и искажает распознавание (Д1): несогласие = предательство.</t>
   </si>
   <si>
-    <t>Катастрофа Challenger; заливы Свиней; корпоративные провалы</t>
+    <t>Катастрофа Challenger; совет, единогласно одобривший провальный план, — сомневающиеся молчали</t>
   </si>
   <si>
     <t>4.2.1, 1.B.12</t>

</xml_diff>